<commit_message>
Hoja Aviso en la plantilla con limitaciones del modelo y descargo de responsabilidad
</commit_message>
<xml_diff>
--- a/plantilla_DCF.xlsx
+++ b/plantilla_DCF.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aviso" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,14 +21,14 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +46,18 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -96,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,25 +124,47 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,6 +530,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>AVISO — Lee esto antes de usar los números</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Este archivo es una herramienta educativa. No es asesoramiento financiero, de inversión ni fiscal, y no es una recomendación de compra o venta. Ninguna decisión de inversión debería basarse en él.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Qué es fiable y qué no:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>• La hoja Datos viene de los reportes 10-K de la SEC (EDGAR). El precio de la acción viene de Yahoo Finance y es del día de la descarga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>• Los supuestos de la hoja Supuestos (celdas amarillas) son ejemplos genéricos, iguales para cualquier empresa. No están adaptados a esta compañía. Cámbialos: el resultado depende más de ellos que de los datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>• Un DCF es extremadamente sensible al WACC y al crecimiento perpetuo. Mira la tabla de sensibilidad al final de la hoja DCF: variaciones de un punto cambian el valor por acción de forma drástica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>• El modelo resta la compensación en acciones (SBC) del flujo y además usa acciones diluidas. Es una postura defendible, pero penaliza dos veces la dilución.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>• El extractor mapea etiquetas contables de la SEC de forma automática. Empresas con estructuras atípicas (múltiples clases de acciones, arrendamientos grandes, adquisiciones recientes) pueden salir mal. Contrasta la hoja Datos con el 10-K original antes de fiarte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Verifica siempre los datos en su fuente original: https://www.sec.gov/edgar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -899,43 +1017,43 @@
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
-      <c r="D11" s="12">
+      <c r="D11" s="35">
         <f>1/(1+Supuestos!$B$16)^D4</f>
         <v/>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="35">
         <f>1/(1+Supuestos!$B$16)^E4</f>
         <v/>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="35">
         <f>1/(1+Supuestos!$B$16)^F4</f>
         <v/>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="35">
         <f>1/(1+Supuestos!$B$16)^G4</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="35">
         <f>1/(1+Supuestos!$B$16)^H4</f>
         <v/>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="35">
         <f>1/(1+Supuestos!$B$16)^I4</f>
         <v/>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="35">
         <f>1/(1+Supuestos!$B$16)^J4</f>
         <v/>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="35">
         <f>1/(1+Supuestos!$B$16)^K4</f>
         <v/>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="35">
         <f>1/(1+Supuestos!$B$16)^L4</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="35">
         <f>1/(1+Supuestos!$B$16)^M4</f>
         <v/>
       </c>
@@ -1105,7 +1223,7 @@
           <t>Acciones diluidas (miles de millones)</t>
         </is>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="36">
         <f>Datos!F14</f>
         <v/>
       </c>
@@ -1116,7 +1234,7 @@
           <t>Valor intrínseco por acción ($)</t>
         </is>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="37">
         <f>B23/B24</f>
         <v/>
       </c>
@@ -1127,7 +1245,7 @@
           <t>Precio con margen de seguridad ($)</t>
         </is>
       </c>
-      <c r="B26" s="15">
+      <c r="B26" s="37">
         <f>B25*(1-Supuestos!B18)</f>
         <v/>
       </c>
@@ -1138,7 +1256,7 @@
           <t>Precio actual ($)</t>
         </is>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="38">
         <f>Supuestos!B6</f>
         <v/>
       </c>
@@ -1149,7 +1267,7 @@
           <t>Valor intrínseco vs. precio actual</t>
         </is>
       </c>
-      <c r="B28" s="17">
+      <c r="B28" s="39">
         <f>IF(B27&gt;0,B25/B27-1,"sin precio")</f>
         <v/>
       </c>
@@ -1167,23 +1285,23 @@
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="B31" s="19">
+      <c r="B31" s="40">
         <f>Supuestos!$B$17+(-0.01)</f>
         <v/>
       </c>
-      <c r="C31" s="19">
+      <c r="C31" s="40">
         <f>Supuestos!$B$17+(-0.005)</f>
         <v/>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="40">
         <f>Supuestos!$B$17+(0)</f>
         <v/>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="40">
         <f>Supuestos!$B$17+(0.005)</f>
         <v/>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="40">
         <f>Supuestos!$B$17+(0.01)</f>
         <v/>
       </c>
@@ -1323,7 +1441,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1381,7 +1499,7 @@
           <t>Precio actual de la acción ($)</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n"/>
+      <c r="B6" s="41" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>← lo rellena la app con el precio del día de descarga</t>
@@ -1394,7 +1512,7 @@
           <t>Tasa libre de riesgo (bono del Tesoro 10 años)</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="42" t="n">
         <v>0.045</v>
       </c>
     </row>
@@ -1414,7 +1532,7 @@
           <t>Prima de riesgo de mercado</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="42" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -1424,7 +1542,7 @@
           <t>Costo del capital (Ke = Rf + Beta x Prima)</t>
         </is>
       </c>
-      <c r="B10" s="26">
+      <c r="B10" s="43">
         <f>B7+B8*B9</f>
         <v/>
       </c>
@@ -1435,7 +1553,7 @@
           <t>Costo de la deuda antes de impuestos</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="42" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -1445,7 +1563,7 @@
           <t>Tasa de impuestos</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="42" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -1477,7 +1595,7 @@
           <t>Peso del capital propio  E / (E + D)</t>
         </is>
       </c>
-      <c r="B15" s="26">
+      <c r="B15" s="43">
         <f>IF(B13+B14&gt;0,B13/(B13+B14),1)</f>
         <v/>
       </c>
@@ -1499,7 +1617,7 @@
           <t>Crecimiento perpetuo (g)</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="42" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -1573,50 +1691,50 @@
           <t>Crecimiento de ingresos</t>
         </is>
       </c>
-      <c r="B22" s="29">
+      <c r="B22" s="44">
         <f>Datos!F6/Datos!E6-1</f>
         <v/>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="44">
         <f>(Datos!F6/Datos!B6)^(1/4)-1</f>
         <v/>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="42" t="n">
         <v>0.12</v>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="42">
         <f>$D22+($M22-$D22)*(E$21-1)/9</f>
         <v/>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="42">
         <f>$D22+($M22-$D22)*(F$21-1)/9</f>
         <v/>
       </c>
-      <c r="G22" s="24">
+      <c r="G22" s="42">
         <f>$D22+($M22-$D22)*(G$21-1)/9</f>
         <v/>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="42">
         <f>$D22+($M22-$D22)*(H$21-1)/9</f>
         <v/>
       </c>
-      <c r="I22" s="24">
+      <c r="I22" s="42">
         <f>$D22+($M22-$D22)*(I$21-1)/9</f>
         <v/>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="42">
         <f>$D22+($M22-$D22)*(J$21-1)/9</f>
         <v/>
       </c>
-      <c r="K22" s="24">
+      <c r="K22" s="42">
         <f>$D22+($M22-$D22)*(K$21-1)/9</f>
         <v/>
       </c>
-      <c r="L22" s="24">
+      <c r="L22" s="42">
         <f>$D22+($M22-$D22)*(L$21-1)/9</f>
         <v/>
       </c>
-      <c r="M22" s="24" t="n">
+      <c r="M22" s="42" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -1626,51 +1744,51 @@
           <t>CFO como % de ingresos</t>
         </is>
       </c>
-      <c r="B23" s="29">
+      <c r="B23" s="44">
         <f>Datos!F7/Datos!F6</f>
         <v/>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="44">
         <f>AVERAGE(Datos!D7/Datos!D6,Datos!E7/Datos!E6,Datos!F7/Datos!F6)</f>
         <v/>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="42">
         <f>ROUND(C23,3)</f>
         <v/>
       </c>
-      <c r="E23" s="24">
+      <c r="E23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="I23" s="24">
+      <c r="I23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="K23" s="24">
+      <c r="K23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="L23" s="24">
+      <c r="L23" s="42">
         <f>$D23</f>
         <v/>
       </c>
-      <c r="M23" s="24">
+      <c r="M23" s="42">
         <f>$D23</f>
         <v/>
       </c>
@@ -1681,51 +1799,51 @@
           <t>Capex + arrendamientos como % de ingresos</t>
         </is>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="44">
         <f>(Datos!F8+Datos!F9)/Datos!F6</f>
         <v/>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="44">
         <f>AVERAGE((Datos!B8+Datos!B9)/Datos!B6,(Datos!C8+Datos!C9)/Datos!C6,(Datos!D8+Datos!D9)/Datos!D6,(Datos!E8+Datos!E9)/Datos!E6)</f>
         <v/>
       </c>
-      <c r="D24" s="24">
+      <c r="D24" s="42">
         <f>ROUND(B24,3)</f>
         <v/>
       </c>
-      <c r="E24" s="24">
+      <c r="E24" s="42">
         <f>IF(E$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(E$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="42">
         <f>IF(F$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(F$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="42">
         <f>IF(G$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(G$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="42">
         <f>IF(H$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(H$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="I24" s="24">
+      <c r="I24" s="42">
         <f>IF(I$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(I$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="J24" s="24">
+      <c r="J24" s="42">
         <f>IF(J$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(J$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="K24" s="24">
+      <c r="K24" s="42">
         <f>IF(K$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(K$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="L24" s="24">
+      <c r="L24" s="42">
         <f>IF(L$21&gt;=$B$26,$M24,$D24+($M24-$D24)*(L$21-1)/($B$26-1))</f>
         <v/>
       </c>
-      <c r="M24" s="24">
+      <c r="M24" s="42">
         <f>ROUND(C24,3)</f>
         <v/>
       </c>
@@ -1736,51 +1854,51 @@
           <t>SBC como % de ingresos</t>
         </is>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="44">
         <f>Datos!F10/Datos!F6</f>
         <v/>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="44">
         <f>AVERAGE(Datos!D10/Datos!D6,Datos!E10/Datos!E6,Datos!F10/Datos!F6)</f>
         <v/>
       </c>
-      <c r="D25" s="24">
+      <c r="D25" s="42">
         <f>ROUND(B25,3)</f>
         <v/>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="J25" s="24">
+      <c r="J25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="K25" s="24">
+      <c r="K25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="L25" s="24">
+      <c r="L25" s="42">
         <f>$D25</f>
         <v/>
       </c>
-      <c r="M25" s="24">
+      <c r="M25" s="42">
         <f>$D25</f>
         <v/>
       </c>
@@ -1807,7 +1925,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Corregir avisos: distinguir supuestos derivados del historico de los genericos
</commit_message>
<xml_diff>
--- a/plantilla_DCF.xlsx
+++ b/plantilla_DCF.xlsx
@@ -567,7 +567,7 @@
     <row r="7">
       <c r="A7" s="32" t="inlineStr">
         <is>
-          <t>• Los supuestos de la hoja Supuestos (celdas amarillas) son ejemplos genéricos, iguales para cualquier empresa. No están adaptados a esta compañía. Cámbialos: el resultado depende más de ellos que de los datos.</t>
+          <t>• En la hoja Supuestos, los márgenes de CFO, capex y SBC (% de ingresos) salen del histórico de esta empresa y los pesos del WACC de su deuda y capitalización. El resto de celdas amarillas (crecimiento 12 % → 4 %, beta, tasa libre de riesgo, prima de mercado, coste de deuda, impuestos, g, margen de seguridad) son valores genéricos, iguales para cualquier empresa. Revísalos: el resultado depende más de ellos que de los datos.</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>• El modelo resta la compensación en acciones (SBC) del flujo y además usa acciones diluidas. Es una postura defendible, pero penaliza dos veces la dilución.</t>
+          <t>• El modelo resta la compensación en acciones (SBC) del flujo y además usa acciones diluidas. Las diluidas recogen concesiones ya otorgadas; la SBC proyectada, sobre todo futuras. Puede haber cierto solapamiento y el modelo no lo separa.</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Los valores amarillos que vienen en la plantilla son EJEMPLOS genéricos: reemplázalos antes de sacar conclusiones.</t>
+          <t>Parte de los valores amarillos (crecimiento, beta, tasas, g, margen) son EJEMPLOS genéricos; los márgenes salen del histórico de la hoja Datos. Revísalos antes de sacar conclusiones.</t>
         </is>
       </c>
     </row>

</xml_diff>